<commit_message>
Completando proceso de Descarga y Consolidacion
</commit_message>
<xml_diff>
--- a/data/raw/rrhh/Colaboradores Migrados a IDM.xlsx
+++ b/data/raw/rrhh/Colaboradores Migrados a IDM.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Universidad\AccesClean\RecursosHumanos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{42CFAEC3-D8DC-48EB-AB03-9517E7FCF08D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494228DD-C4E0-45B3-B594-C5CD3ABD9C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AAB666E4-D677-439C-B12F-F6651931957C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$S$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>